<commit_message>
Fix platform login: add missing platform_users auth columns + tags fixes
- platformAuth.controller queried password_hash/lockout columns that
  migration 020 never created — every /platform/login attempt 500'd.
  Migration 073 adds them; admin@kmaincms.org seeded with dev password.
- Migration 072 creates payment_receipt_counters + document_tags
  (referenced by pending repository changes) with jsonb-aware backfill.
- DocumentsRepository: tags is jsonb — raw JS arrays failed the cast
  (invalid input syntax for type json); normalize to JSON strings and
  sync the document_tags junction via unnest.

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/plans/2026-10-03_test-credentials.xlsx
+++ b/docs/plans/2026-10-03_test-credentials.xlsx
@@ -95,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -109,6 +109,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -474,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1874,6 +1875,38 @@
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Platform Console</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Platform Owner</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>admin@kmaincms.org</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>admin@kmaincms.org</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>right123</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>Separate login page: /platform/login</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:F50"/>
@@ -1890,7 +1923,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2266,6 +2299,33 @@
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Platform Console</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>admin@kmaincms.org</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>admin@kmaincms.org</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>right123</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Separate login page: /platform/login — different user table</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3296,7 +3356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3418,6 +3478,18 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Platform login</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>admin@kmaincms.org / right123 works ONLY at /platform/login (the platform console). The normal /auth/login form uses the church users table — superadmin there is username superadmin / right123.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>